<commit_message>
WorkLog done, here we go!
</commit_message>
<xml_diff>
--- a/Block B/Worklog - Y1B-2024-25_ADSAI.xlsx
+++ b/Block B/Worklog - Y1B-2024-25_ADSAI.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Deliverables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maksb\Documents\GitHub\2024-25b-fai1-adsai-MaksBurchard240894\Block B\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C4FA678-DBF0-4070-BD9B-7756FAE36615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E25633F1-EE2E-4C73-AB43-0477F4CAB7BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1433" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1447" uniqueCount="420">
   <si>
     <t>Date</t>
   </si>
@@ -1199,9 +1199,6 @@
     <t>https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/tree/0e7620868343501c8dfcfa39189c1d60ae3a3b5e/Old%20Python%20Files</t>
   </si>
   <si>
-    <t>AAA</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894 </t>
   </si>
   <si>
@@ -1223,9 +1220,6 @@
     <t>I had the content fresh in my mind so I did this quicker than expected.</t>
   </si>
   <si>
-    <t>I'm still not too sure about the SMATER goals. AAA</t>
-  </si>
-  <si>
     <t>https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/blob/0e7620868343501c8dfcfa39189c1d60ae3a3b5e/Block%20B/2024-11-25.png</t>
   </si>
   <si>
@@ -1350,6 +1344,24 @@
   </si>
   <si>
     <t>Finish Learning Log section C</t>
+  </si>
+  <si>
+    <t>Finish Learning Log section D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/blob/fb4c74bf2f88e2d2d88a4f4e5bd1c705b0ee03bc/Deliverables/Worklog%20-%20Y1B-2024-25_ADSAI.xlsx </t>
+  </si>
+  <si>
+    <t>Self-refrence finished WorkLog &amp; Learning Log in WorkLog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/BredaUniversityADSAI/2024-25b-fai1-adsai-MaksBurchard240894/blob/fb4c74bf2f88e2d2d88a4f4e5bd1c705b0ee03bc/Deliverables/Learning%20Log%20-%20Y1B-2024-25_ADSAI.pptx </t>
+  </si>
+  <si>
+    <t>See this document</t>
+  </si>
+  <si>
+    <t>I'm still not too sure about the SMATER goals.</t>
   </si>
 </sst>
 </file>
@@ -1845,6 +1857,26 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1861,8 +1893,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1880,24 +1910,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2322,7 +2334,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K264"/>
+  <dimension ref="A1:K266"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.90625" customWidth="1"/>
@@ -2374,53 +2386,53 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="68" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="61"/>
-      <c r="C2" s="61"/>
-      <c r="D2" s="61"/>
-      <c r="E2" s="61"/>
-      <c r="F2" s="61"/>
-      <c r="G2" s="61"/>
-      <c r="H2" s="61"/>
-      <c r="I2" s="61"/>
-      <c r="J2" s="61"/>
-      <c r="K2" s="62"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="70"/>
     </row>
     <row r="3" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="63" t="s">
+      <c r="B3" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
-      <c r="K3" s="65"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="58"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="63" t="s">
+      <c r="B4" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="64"/>
-      <c r="D4" s="64"/>
-      <c r="E4" s="64"/>
-      <c r="F4" s="64"/>
-      <c r="G4" s="64"/>
-      <c r="H4" s="64"/>
-      <c r="I4" s="64"/>
-      <c r="J4" s="64"/>
-      <c r="K4" s="65"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="57"/>
+      <c r="H4" s="57"/>
+      <c r="I4" s="57"/>
+      <c r="J4" s="57"/>
+      <c r="K4" s="58"/>
     </row>
     <row r="5" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="37">
@@ -2550,7 +2562,7 @@
         <v>-0.5</v>
       </c>
       <c r="J8" s="53" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="K8" s="44"/>
     </row>
@@ -2684,7 +2696,7 @@
         <v>-0.25</v>
       </c>
       <c r="J12" s="53" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="K12" s="44"/>
     </row>
@@ -2750,7 +2762,7 @@
         <v>0</v>
       </c>
       <c r="J14" s="53" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="K14" s="44"/>
     </row>
@@ -2783,10 +2795,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J15" s="45"/>
-      <c r="K15" s="44" t="s">
-        <v>365</v>
-      </c>
+      <c r="J15" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K15" s="44"/>
     </row>
     <row r="16" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A16" s="37">
@@ -2818,7 +2830,7 @@
         <v>0</v>
       </c>
       <c r="J16" s="53" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="K16" s="44"/>
     </row>
@@ -2853,7 +2865,7 @@
       </c>
       <c r="J17" s="45"/>
       <c r="K17" s="44" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -2885,10 +2897,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J18" s="45"/>
-      <c r="K18" s="44" t="s">
-        <v>365</v>
-      </c>
+      <c r="J18" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K18" s="44"/>
     </row>
     <row r="19" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A19" s="37">
@@ -2969,7 +2981,7 @@
         <v>227</v>
       </c>
       <c r="D21" s="38" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E21" s="40" t="s">
         <v>49</v>
@@ -2988,7 +3000,7 @@
         <v>0</v>
       </c>
       <c r="J21" s="53" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="K21" s="44"/>
     </row>
@@ -3053,10 +3065,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J23" s="45"/>
-      <c r="K23" s="44" t="s">
-        <v>365</v>
-      </c>
+      <c r="J23" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K23" s="44"/>
     </row>
     <row r="24" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A24" s="37">
@@ -3088,7 +3100,7 @@
         <v>0</v>
       </c>
       <c r="J24" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K24" s="44"/>
     </row>
@@ -3122,7 +3134,7 @@
         <v>0</v>
       </c>
       <c r="J25" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K25" s="44"/>
     </row>
@@ -3156,7 +3168,7 @@
         <v>0</v>
       </c>
       <c r="J26" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K26" s="44"/>
     </row>
@@ -3190,7 +3202,7 @@
         <v>0</v>
       </c>
       <c r="J27" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K27" s="44"/>
     </row>
@@ -3224,7 +3236,7 @@
         <v>0</v>
       </c>
       <c r="J28" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K28" s="44"/>
     </row>
@@ -3261,7 +3273,7 @@
         <v>105</v>
       </c>
       <c r="K29" s="44" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -3294,7 +3306,7 @@
         <v>0</v>
       </c>
       <c r="J30" s="53" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="K30" s="44"/>
     </row>
@@ -3327,10 +3339,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J31" s="45"/>
-      <c r="K31" s="44" t="s">
-        <v>365</v>
-      </c>
+      <c r="J31" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K31" s="44"/>
     </row>
     <row r="32" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A32" s="37">
@@ -3556,7 +3568,7 @@
         <v>0</v>
       </c>
       <c r="J38" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K38" s="44"/>
     </row>
@@ -3590,7 +3602,7 @@
         <v>0</v>
       </c>
       <c r="J39" s="53" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="K39" s="44" t="s">
         <v>139</v>
@@ -3626,7 +3638,7 @@
         <v>0</v>
       </c>
       <c r="J40" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K40" s="44"/>
     </row>
@@ -3659,10 +3671,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J41" s="45"/>
-      <c r="K41" s="44" t="s">
-        <v>365</v>
-      </c>
+      <c r="J41" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K41" s="44"/>
     </row>
     <row r="42" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A42" s="37">
@@ -3693,7 +3705,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J42" s="45"/>
+      <c r="J42" s="53" t="s">
+        <v>417</v>
+      </c>
       <c r="K42" s="44"/>
     </row>
     <row r="43" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -3725,10 +3739,10 @@
         <f t="shared" si="0"/>
         <v>-0.35</v>
       </c>
-      <c r="J43" s="45"/>
-      <c r="K43" s="44" t="s">
-        <v>365</v>
-      </c>
+      <c r="J43" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K43" s="44"/>
     </row>
     <row r="44" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A44" s="13"/>
@@ -3755,53 +3769,53 @@
       <c r="K44" s="46"/>
     </row>
     <row r="45" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="66" t="s">
+      <c r="A45" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="B45" s="61"/>
-      <c r="C45" s="61"/>
-      <c r="D45" s="61"/>
-      <c r="E45" s="61"/>
-      <c r="F45" s="61"/>
-      <c r="G45" s="61"/>
-      <c r="H45" s="61"/>
-      <c r="I45" s="61"/>
-      <c r="J45" s="61"/>
-      <c r="K45" s="62"/>
+      <c r="B45" s="69"/>
+      <c r="C45" s="69"/>
+      <c r="D45" s="69"/>
+      <c r="E45" s="69"/>
+      <c r="F45" s="69"/>
+      <c r="G45" s="69"/>
+      <c r="H45" s="69"/>
+      <c r="I45" s="69"/>
+      <c r="J45" s="69"/>
+      <c r="K45" s="70"/>
     </row>
     <row r="46" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A46" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B46" s="67" t="s">
+      <c r="B46" s="73" t="s">
         <v>13</v>
       </c>
-      <c r="C46" s="64"/>
-      <c r="D46" s="64"/>
-      <c r="E46" s="64"/>
-      <c r="F46" s="64"/>
-      <c r="G46" s="64"/>
-      <c r="H46" s="64"/>
-      <c r="I46" s="64"/>
-      <c r="J46" s="64"/>
-      <c r="K46" s="65"/>
+      <c r="C46" s="57"/>
+      <c r="D46" s="57"/>
+      <c r="E46" s="57"/>
+      <c r="F46" s="57"/>
+      <c r="G46" s="57"/>
+      <c r="H46" s="57"/>
+      <c r="I46" s="57"/>
+      <c r="J46" s="57"/>
+      <c r="K46" s="58"/>
     </row>
     <row r="47" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B47" s="67" t="s">
+      <c r="B47" s="73" t="s">
         <v>20</v>
       </c>
-      <c r="C47" s="64"/>
-      <c r="D47" s="64"/>
-      <c r="E47" s="64"/>
-      <c r="F47" s="64"/>
-      <c r="G47" s="64"/>
-      <c r="H47" s="64"/>
-      <c r="I47" s="64"/>
-      <c r="J47" s="64"/>
-      <c r="K47" s="65"/>
+      <c r="C47" s="57"/>
+      <c r="D47" s="57"/>
+      <c r="E47" s="57"/>
+      <c r="F47" s="57"/>
+      <c r="G47" s="57"/>
+      <c r="H47" s="57"/>
+      <c r="I47" s="57"/>
+      <c r="J47" s="57"/>
+      <c r="K47" s="58"/>
     </row>
     <row r="48" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A48" s="47">
@@ -3832,10 +3846,10 @@
         <f t="shared" ref="I48:I79" si="1">H48-G48</f>
         <v>0</v>
       </c>
-      <c r="J48" s="45"/>
-      <c r="K48" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J48" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K48" s="43"/>
     </row>
     <row r="49" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A49" s="47">
@@ -3867,7 +3881,7 @@
         <v>0</v>
       </c>
       <c r="J49" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K49" s="43"/>
     </row>
@@ -3901,7 +3915,7 @@
         <v>0</v>
       </c>
       <c r="J50" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K50" s="43"/>
     </row>
@@ -3935,7 +3949,7 @@
         <v>0</v>
       </c>
       <c r="J51" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K51" s="43"/>
     </row>
@@ -3969,7 +3983,7 @@
         <v>0</v>
       </c>
       <c r="J52" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K52" s="43"/>
     </row>
@@ -4003,7 +4017,7 @@
         <v>0</v>
       </c>
       <c r="J53" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K53" s="43"/>
     </row>
@@ -4037,7 +4051,7 @@
         <v>0</v>
       </c>
       <c r="J54" s="53" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="K54" s="43"/>
     </row>
@@ -4070,10 +4084,10 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J55" s="45"/>
-      <c r="K55" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J55" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K55" s="43"/>
     </row>
     <row r="56" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A56" s="47">
@@ -4171,7 +4185,7 @@
         <v>0</v>
       </c>
       <c r="J58" s="53" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="K58" s="43"/>
     </row>
@@ -4307,7 +4321,7 @@
         <v>-0.45000000000000018</v>
       </c>
       <c r="J62" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K62" s="43"/>
     </row>
@@ -4405,7 +4419,7 @@
         <v>0</v>
       </c>
       <c r="J65" s="53" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="K65" s="43"/>
     </row>
@@ -4471,7 +4485,7 @@
         <v>-0.25</v>
       </c>
       <c r="J67" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K67" s="43"/>
     </row>
@@ -4633,7 +4647,7 @@
         <v>-0.5</v>
       </c>
       <c r="J72" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K72" s="43"/>
     </row>
@@ -4698,10 +4712,10 @@
         <f>H74-G74</f>
         <v>0</v>
       </c>
-      <c r="J74" s="45"/>
-      <c r="K74" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J74" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K74" s="43"/>
     </row>
     <row r="75" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A75" s="47">
@@ -4732,9 +4746,11 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J75" s="45"/>
+      <c r="J75" s="53" t="s">
+        <v>417</v>
+      </c>
       <c r="K75" s="43" t="s">
-        <v>373</v>
+        <v>419</v>
       </c>
     </row>
     <row r="76" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -4766,10 +4782,10 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J76" s="45"/>
-      <c r="K76" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J76" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K76" s="43"/>
     </row>
     <row r="77" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A77" s="47">
@@ -4800,10 +4816,10 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J77" s="45"/>
-      <c r="K77" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J77" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K77" s="43"/>
     </row>
     <row r="78" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A78" s="47">
@@ -4834,10 +4850,10 @@
         <f t="shared" si="1"/>
         <v>-0.1</v>
       </c>
-      <c r="J78" s="45"/>
-      <c r="K78" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J78" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K78" s="43"/>
     </row>
     <row r="79" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A79" s="13"/>
@@ -4864,53 +4880,53 @@
       <c r="K79" s="46"/>
     </row>
     <row r="80" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="68" t="s">
+      <c r="A80" s="74" t="s">
         <v>21</v>
       </c>
-      <c r="B80" s="64"/>
-      <c r="C80" s="64"/>
-      <c r="D80" s="64"/>
-      <c r="E80" s="64"/>
-      <c r="F80" s="64"/>
-      <c r="G80" s="64"/>
-      <c r="H80" s="64"/>
-      <c r="I80" s="64"/>
-      <c r="J80" s="64"/>
-      <c r="K80" s="65"/>
+      <c r="B80" s="57"/>
+      <c r="C80" s="57"/>
+      <c r="D80" s="57"/>
+      <c r="E80" s="57"/>
+      <c r="F80" s="57"/>
+      <c r="G80" s="57"/>
+      <c r="H80" s="57"/>
+      <c r="I80" s="57"/>
+      <c r="J80" s="57"/>
+      <c r="K80" s="58"/>
     </row>
     <row r="81" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A81" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B81" s="69" t="s">
+      <c r="B81" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C81" s="64"/>
-      <c r="D81" s="64"/>
-      <c r="E81" s="64"/>
-      <c r="F81" s="64"/>
-      <c r="G81" s="64"/>
-      <c r="H81" s="64"/>
-      <c r="I81" s="64"/>
-      <c r="J81" s="64"/>
-      <c r="K81" s="65"/>
+      <c r="C81" s="57"/>
+      <c r="D81" s="57"/>
+      <c r="E81" s="57"/>
+      <c r="F81" s="57"/>
+      <c r="G81" s="57"/>
+      <c r="H81" s="57"/>
+      <c r="I81" s="57"/>
+      <c r="J81" s="57"/>
+      <c r="K81" s="58"/>
     </row>
     <row r="82" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B82" s="69" t="s">
+      <c r="B82" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="C82" s="64"/>
-      <c r="D82" s="64"/>
-      <c r="E82" s="64"/>
-      <c r="F82" s="64"/>
-      <c r="G82" s="64"/>
-      <c r="H82" s="64"/>
-      <c r="I82" s="64"/>
-      <c r="J82" s="64"/>
-      <c r="K82" s="65"/>
+      <c r="C82" s="57"/>
+      <c r="D82" s="57"/>
+      <c r="E82" s="57"/>
+      <c r="F82" s="57"/>
+      <c r="G82" s="57"/>
+      <c r="H82" s="57"/>
+      <c r="I82" s="57"/>
+      <c r="J82" s="57"/>
+      <c r="K82" s="58"/>
     </row>
     <row r="83" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A83" s="37">
@@ -4941,10 +4957,10 @@
         <f t="shared" ref="I83:I113" si="2">H83-G83</f>
         <v>0</v>
       </c>
-      <c r="J83" s="45"/>
-      <c r="K83" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J83" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K83" s="43"/>
     </row>
     <row r="84" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A84" s="37">
@@ -4975,10 +4991,10 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J84" s="45"/>
-      <c r="K84" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J84" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K84" s="43"/>
     </row>
     <row r="85" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A85" s="37">
@@ -5010,7 +5026,7 @@
         <v>-0.5</v>
       </c>
       <c r="J85" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K85" s="43"/>
     </row>
@@ -5076,7 +5092,7 @@
         <v>-0.25</v>
       </c>
       <c r="J87" s="53" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="K87" s="43"/>
     </row>
@@ -5110,7 +5126,7 @@
         <v>-1</v>
       </c>
       <c r="J88" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K88" s="43"/>
     </row>
@@ -5176,7 +5192,7 @@
         <v>0.5</v>
       </c>
       <c r="J90" s="53" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="K90" s="43" t="s">
         <v>156</v>
@@ -5243,10 +5259,10 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J92" s="45"/>
-      <c r="K92" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J92" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K92" s="43"/>
     </row>
     <row r="93" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A93" s="37">
@@ -5310,7 +5326,7 @@
         <v>1.5</v>
       </c>
       <c r="J94" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K94" s="43" t="s">
         <v>163</v>
@@ -5346,7 +5362,7 @@
         <v>0</v>
       </c>
       <c r="J95" s="53" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="K95" s="43"/>
     </row>
@@ -5380,7 +5396,7 @@
         <v>-0.5</v>
       </c>
       <c r="J96" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K96" s="43"/>
     </row>
@@ -5447,7 +5463,7 @@
       </c>
       <c r="J98" s="45"/>
       <c r="K98" s="43" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="99" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -5480,7 +5496,7 @@
         <v>0</v>
       </c>
       <c r="J99" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K99" s="43"/>
     </row>
@@ -5514,7 +5530,7 @@
         <v>0</v>
       </c>
       <c r="J100" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K100" s="43"/>
     </row>
@@ -5548,7 +5564,7 @@
         <v>0</v>
       </c>
       <c r="J101" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K101" s="43"/>
     </row>
@@ -5582,7 +5598,7 @@
         <v>0</v>
       </c>
       <c r="J102" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K102" s="43"/>
     </row>
@@ -5616,7 +5632,7 @@
         <v>0</v>
       </c>
       <c r="J103" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K103" s="43"/>
     </row>
@@ -5714,7 +5730,7 @@
         <v>0</v>
       </c>
       <c r="J106" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K106" s="43"/>
     </row>
@@ -5780,7 +5796,7 @@
         <v>-1</v>
       </c>
       <c r="J108" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K108" s="43" t="s">
         <v>198</v>
@@ -5815,10 +5831,10 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J109" s="45"/>
-      <c r="K109" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J109" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K109" s="43"/>
     </row>
     <row r="110" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A110" s="37">
@@ -5849,10 +5865,10 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J110" s="45"/>
-      <c r="K110" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J110" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K110" s="43"/>
     </row>
     <row r="111" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A111" s="37">
@@ -5883,10 +5899,10 @@
         <f t="shared" si="2"/>
         <v>-0.25</v>
       </c>
-      <c r="J111" s="45"/>
-      <c r="K111" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J111" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K111" s="43"/>
     </row>
     <row r="112" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A112" s="37">
@@ -5917,10 +5933,10 @@
         <f t="shared" si="2"/>
         <v>-0.25</v>
       </c>
-      <c r="J112" s="45"/>
-      <c r="K112" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J112" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K112" s="43"/>
     </row>
     <row r="113" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A113" s="13"/>
@@ -5947,53 +5963,53 @@
       <c r="K113" s="46"/>
     </row>
     <row r="114" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="70" t="s">
+      <c r="A114" s="76" t="s">
         <v>22</v>
       </c>
-      <c r="B114" s="64"/>
-      <c r="C114" s="64"/>
-      <c r="D114" s="64"/>
-      <c r="E114" s="64"/>
-      <c r="F114" s="64"/>
-      <c r="G114" s="64"/>
-      <c r="H114" s="64"/>
-      <c r="I114" s="64"/>
-      <c r="J114" s="64"/>
-      <c r="K114" s="65"/>
+      <c r="B114" s="57"/>
+      <c r="C114" s="57"/>
+      <c r="D114" s="57"/>
+      <c r="E114" s="57"/>
+      <c r="F114" s="57"/>
+      <c r="G114" s="57"/>
+      <c r="H114" s="57"/>
+      <c r="I114" s="57"/>
+      <c r="J114" s="57"/>
+      <c r="K114" s="58"/>
     </row>
     <row r="115" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A115" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B115" s="72" t="s">
+      <c r="B115" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="C115" s="64"/>
-      <c r="D115" s="64"/>
-      <c r="E115" s="64"/>
-      <c r="F115" s="64"/>
-      <c r="G115" s="64"/>
-      <c r="H115" s="64"/>
-      <c r="I115" s="64"/>
-      <c r="J115" s="64"/>
-      <c r="K115" s="65"/>
+      <c r="C115" s="57"/>
+      <c r="D115" s="57"/>
+      <c r="E115" s="57"/>
+      <c r="F115" s="57"/>
+      <c r="G115" s="57"/>
+      <c r="H115" s="57"/>
+      <c r="I115" s="57"/>
+      <c r="J115" s="57"/>
+      <c r="K115" s="58"/>
     </row>
     <row r="116" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B116" s="72" t="s">
+      <c r="B116" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="C116" s="64"/>
-      <c r="D116" s="64"/>
-      <c r="E116" s="64"/>
-      <c r="F116" s="64"/>
-      <c r="G116" s="64"/>
-      <c r="H116" s="64"/>
-      <c r="I116" s="64"/>
-      <c r="J116" s="64"/>
-      <c r="K116" s="65"/>
+      <c r="C116" s="57"/>
+      <c r="D116" s="57"/>
+      <c r="E116" s="57"/>
+      <c r="F116" s="57"/>
+      <c r="G116" s="57"/>
+      <c r="H116" s="57"/>
+      <c r="I116" s="57"/>
+      <c r="J116" s="57"/>
+      <c r="K116" s="58"/>
     </row>
     <row r="117" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A117" s="37">
@@ -6024,10 +6040,10 @@
         <f t="shared" ref="I117:I118" si="3">H117-G117</f>
         <v>0</v>
       </c>
-      <c r="J117" s="45"/>
-      <c r="K117" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J117" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K117" s="43"/>
     </row>
     <row r="118" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A118" s="37">
@@ -6058,10 +6074,10 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="J118" s="45"/>
-      <c r="K118" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J118" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K118" s="43"/>
     </row>
     <row r="119" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A119" s="37">
@@ -6093,7 +6109,7 @@
         <v>0</v>
       </c>
       <c r="J119" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K119" s="43"/>
     </row>
@@ -6127,7 +6143,7 @@
         <v>-0.5</v>
       </c>
       <c r="J120" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K120" s="43"/>
     </row>
@@ -6161,7 +6177,7 @@
         <v>-0.5</v>
       </c>
       <c r="J121" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K121" s="43"/>
     </row>
@@ -6195,7 +6211,7 @@
         <v>-0.5</v>
       </c>
       <c r="J122" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K122" s="43"/>
     </row>
@@ -6229,7 +6245,7 @@
         <v>-0.5</v>
       </c>
       <c r="J123" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K123" s="43"/>
     </row>
@@ -6295,7 +6311,7 @@
         <v>0</v>
       </c>
       <c r="J125" s="53" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="K125" s="43"/>
     </row>
@@ -6363,7 +6379,7 @@
         <v>0</v>
       </c>
       <c r="J127" s="53" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="K127" s="43"/>
     </row>
@@ -6429,7 +6445,7 @@
         <v>-0.5</v>
       </c>
       <c r="J129" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K129" s="43"/>
     </row>
@@ -6463,7 +6479,7 @@
         <v>-0.5</v>
       </c>
       <c r="J130" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K130" s="43"/>
     </row>
@@ -6497,7 +6513,7 @@
         <v>-0.5</v>
       </c>
       <c r="J131" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K131" s="43"/>
     </row>
@@ -6531,7 +6547,7 @@
         <v>-0.5</v>
       </c>
       <c r="J132" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K132" s="43"/>
     </row>
@@ -6565,7 +6581,7 @@
         <v>-0.5</v>
       </c>
       <c r="J133" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K133" s="43"/>
     </row>
@@ -6631,7 +6647,7 @@
         <v>0</v>
       </c>
       <c r="J135" s="53" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="K135" s="43"/>
     </row>
@@ -6697,10 +6713,10 @@
         <v>-1</v>
       </c>
       <c r="J137" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K137" s="43" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="138" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -6732,10 +6748,10 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J138" s="45"/>
-      <c r="K138" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J138" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K138" s="43"/>
     </row>
     <row r="139" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A139" s="37">
@@ -6831,7 +6847,7 @@
         <v>0</v>
       </c>
       <c r="J141" s="53" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="K141" s="43"/>
     </row>
@@ -6865,7 +6881,7 @@
         <v>0</v>
       </c>
       <c r="J142" s="53" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="K142" s="43"/>
     </row>
@@ -6898,10 +6914,10 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J143" s="45"/>
-      <c r="K143" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J143" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K143" s="43"/>
     </row>
     <row r="144" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A144" s="37">
@@ -6932,10 +6948,10 @@
         <f t="shared" si="4"/>
         <v>-0.25</v>
       </c>
-      <c r="J144" s="45"/>
-      <c r="K144" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J144" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K144" s="43"/>
     </row>
     <row r="145" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A145" s="37">
@@ -6966,10 +6982,10 @@
         <f t="shared" si="4"/>
         <v>-0.25</v>
       </c>
-      <c r="J145" s="45"/>
-      <c r="K145" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J145" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K145" s="43"/>
     </row>
     <row r="146" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A146" s="13"/>
@@ -6996,53 +7012,53 @@
       <c r="K146" s="46"/>
     </row>
     <row r="147" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A147" s="75" t="s">
+      <c r="A147" s="61" t="s">
         <v>23</v>
       </c>
-      <c r="B147" s="64"/>
-      <c r="C147" s="64"/>
-      <c r="D147" s="64"/>
-      <c r="E147" s="64"/>
-      <c r="F147" s="64"/>
-      <c r="G147" s="64"/>
-      <c r="H147" s="64"/>
-      <c r="I147" s="64"/>
-      <c r="J147" s="64"/>
-      <c r="K147" s="65"/>
+      <c r="B147" s="57"/>
+      <c r="C147" s="57"/>
+      <c r="D147" s="57"/>
+      <c r="E147" s="57"/>
+      <c r="F147" s="57"/>
+      <c r="G147" s="57"/>
+      <c r="H147" s="57"/>
+      <c r="I147" s="57"/>
+      <c r="J147" s="57"/>
+      <c r="K147" s="58"/>
     </row>
     <row r="148" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A148" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B148" s="76" t="s">
+      <c r="B148" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="C148" s="64"/>
-      <c r="D148" s="64"/>
-      <c r="E148" s="64"/>
-      <c r="F148" s="64"/>
-      <c r="G148" s="64"/>
-      <c r="H148" s="64"/>
-      <c r="I148" s="64"/>
-      <c r="J148" s="64"/>
-      <c r="K148" s="65"/>
+      <c r="C148" s="57"/>
+      <c r="D148" s="57"/>
+      <c r="E148" s="57"/>
+      <c r="F148" s="57"/>
+      <c r="G148" s="57"/>
+      <c r="H148" s="57"/>
+      <c r="I148" s="57"/>
+      <c r="J148" s="57"/>
+      <c r="K148" s="58"/>
     </row>
     <row r="149" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B149" s="76" t="s">
+      <c r="B149" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="C149" s="64"/>
-      <c r="D149" s="64"/>
-      <c r="E149" s="64"/>
-      <c r="F149" s="64"/>
-      <c r="G149" s="64"/>
-      <c r="H149" s="64"/>
-      <c r="I149" s="64"/>
-      <c r="J149" s="64"/>
-      <c r="K149" s="65"/>
+      <c r="C149" s="57"/>
+      <c r="D149" s="57"/>
+      <c r="E149" s="57"/>
+      <c r="F149" s="57"/>
+      <c r="G149" s="57"/>
+      <c r="H149" s="57"/>
+      <c r="I149" s="57"/>
+      <c r="J149" s="57"/>
+      <c r="K149" s="58"/>
     </row>
     <row r="150" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A150" s="37">
@@ -7073,10 +7089,10 @@
         <f t="shared" ref="I150:I189" si="5">H150-G150</f>
         <v>0</v>
       </c>
-      <c r="J150" s="45"/>
-      <c r="K150" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J150" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K150" s="43"/>
     </row>
     <row r="151" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A151" s="37">
@@ -7107,10 +7123,10 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J151" s="45"/>
-      <c r="K151" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J151" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K151" s="43"/>
     </row>
     <row r="152" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A152" s="37">
@@ -7142,7 +7158,7 @@
         <v>0</v>
       </c>
       <c r="J152" s="53" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="K152" s="43"/>
     </row>
@@ -7208,7 +7224,7 @@
         <v>-0.5</v>
       </c>
       <c r="J154" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K154" s="43"/>
     </row>
@@ -7242,7 +7258,7 @@
         <v>-0.5</v>
       </c>
       <c r="J155" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K155" s="43"/>
     </row>
@@ -7276,7 +7292,7 @@
         <v>-0.5</v>
       </c>
       <c r="J156" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K156" s="43"/>
     </row>
@@ -7310,7 +7326,7 @@
         <v>-0.5</v>
       </c>
       <c r="J157" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K157" s="43"/>
     </row>
@@ -7376,7 +7392,7 @@
         <v>-0.25</v>
       </c>
       <c r="J159" s="53" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="K159" s="43"/>
     </row>
@@ -7442,7 +7458,7 @@
         <v>-0.5</v>
       </c>
       <c r="J161" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K161" s="43"/>
     </row>
@@ -7476,7 +7492,7 @@
         <v>-1</v>
       </c>
       <c r="J162" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K162" s="43"/>
     </row>
@@ -7510,7 +7526,7 @@
         <v>-1</v>
       </c>
       <c r="J163" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K163" s="43"/>
     </row>
@@ -7544,7 +7560,7 @@
         <v>-1</v>
       </c>
       <c r="J164" s="53" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K164" s="43"/>
     </row>
@@ -7610,7 +7626,7 @@
         <v>0</v>
       </c>
       <c r="J166" s="53" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="K166" s="43"/>
     </row>
@@ -7643,10 +7659,10 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J167" s="45"/>
-      <c r="K167" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J167" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K167" s="43"/>
     </row>
     <row r="168" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A168" s="37">
@@ -7709,10 +7725,10 @@
         <f t="shared" si="5"/>
         <v>-0.5</v>
       </c>
-      <c r="J169" s="45"/>
-      <c r="K169" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J169" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K169" s="43"/>
     </row>
     <row r="170" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A170" s="37">
@@ -7744,7 +7760,7 @@
         <v>0</v>
       </c>
       <c r="J170" s="53" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="K170" s="43"/>
     </row>
@@ -7778,7 +7794,7 @@
         <v>0.5</v>
       </c>
       <c r="J171" s="53" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="K171" s="43" t="s">
         <v>267</v>
@@ -7814,7 +7830,7 @@
         <v>0</v>
       </c>
       <c r="J172" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K172" s="43"/>
     </row>
@@ -7848,7 +7864,7 @@
         <v>0</v>
       </c>
       <c r="J173" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K173" s="43"/>
     </row>
@@ -7916,7 +7932,7 @@
         <v>-0.25</v>
       </c>
       <c r="J175" s="53" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="K175" s="43" t="s">
         <v>273</v>
@@ -7983,10 +7999,10 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J177" s="45"/>
-      <c r="K177" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J177" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K177" s="43"/>
     </row>
     <row r="178" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A178" s="37">
@@ -8050,7 +8066,7 @@
         <v>2.25</v>
       </c>
       <c r="J179" s="53" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="K179" s="43" t="s">
         <v>325</v>
@@ -8118,7 +8134,7 @@
         <v>0</v>
       </c>
       <c r="J181" s="53" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="K181" s="43"/>
     </row>
@@ -8152,7 +8168,7 @@
         <v>0</v>
       </c>
       <c r="J182" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K182" s="43"/>
     </row>
@@ -8186,7 +8202,7 @@
         <v>0</v>
       </c>
       <c r="J183" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K183" s="43"/>
     </row>
@@ -8220,7 +8236,7 @@
         <v>0</v>
       </c>
       <c r="J184" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K184" s="43"/>
     </row>
@@ -8253,10 +8269,10 @@
         <f t="shared" si="5"/>
         <v>-0.1</v>
       </c>
-      <c r="J185" s="45"/>
-      <c r="K185" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J185" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K185" s="43"/>
     </row>
     <row r="186" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A186" s="37">
@@ -8287,10 +8303,10 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J186" s="45"/>
-      <c r="K186" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J186" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K186" s="43"/>
     </row>
     <row r="187" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A187" s="37">
@@ -8321,10 +8337,10 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J187" s="45"/>
-      <c r="K187" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J187" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K187" s="43"/>
     </row>
     <row r="188" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A188" s="37">
@@ -8355,10 +8371,10 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J188" s="45"/>
-      <c r="K188" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J188" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K188" s="43"/>
     </row>
     <row r="189" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A189" s="13"/>
@@ -8385,53 +8401,53 @@
       <c r="K189" s="46"/>
     </row>
     <row r="190" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A190" s="77" t="s">
+      <c r="A190" s="63" t="s">
         <v>24</v>
       </c>
-      <c r="B190" s="64"/>
-      <c r="C190" s="64"/>
-      <c r="D190" s="64"/>
-      <c r="E190" s="64"/>
-      <c r="F190" s="64"/>
-      <c r="G190" s="64"/>
-      <c r="H190" s="64"/>
-      <c r="I190" s="64"/>
-      <c r="J190" s="64"/>
-      <c r="K190" s="65"/>
+      <c r="B190" s="57"/>
+      <c r="C190" s="57"/>
+      <c r="D190" s="57"/>
+      <c r="E190" s="57"/>
+      <c r="F190" s="57"/>
+      <c r="G190" s="57"/>
+      <c r="H190" s="57"/>
+      <c r="I190" s="57"/>
+      <c r="J190" s="57"/>
+      <c r="K190" s="58"/>
     </row>
     <row r="191" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A191" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B191" s="73" t="s">
+      <c r="B191" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="C191" s="64"/>
-      <c r="D191" s="64"/>
-      <c r="E191" s="64"/>
-      <c r="F191" s="64"/>
-      <c r="G191" s="64"/>
-      <c r="H191" s="64"/>
-      <c r="I191" s="64"/>
-      <c r="J191" s="64"/>
-      <c r="K191" s="65"/>
+      <c r="C191" s="57"/>
+      <c r="D191" s="57"/>
+      <c r="E191" s="57"/>
+      <c r="F191" s="57"/>
+      <c r="G191" s="57"/>
+      <c r="H191" s="57"/>
+      <c r="I191" s="57"/>
+      <c r="J191" s="57"/>
+      <c r="K191" s="58"/>
     </row>
     <row r="192" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B192" s="73" t="s">
+      <c r="B192" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="C192" s="64"/>
-      <c r="D192" s="64"/>
-      <c r="E192" s="64"/>
-      <c r="F192" s="64"/>
-      <c r="G192" s="64"/>
-      <c r="H192" s="64"/>
-      <c r="I192" s="64"/>
-      <c r="J192" s="64"/>
-      <c r="K192" s="65"/>
+      <c r="C192" s="57"/>
+      <c r="D192" s="57"/>
+      <c r="E192" s="57"/>
+      <c r="F192" s="57"/>
+      <c r="G192" s="57"/>
+      <c r="H192" s="57"/>
+      <c r="I192" s="57"/>
+      <c r="J192" s="57"/>
+      <c r="K192" s="58"/>
     </row>
     <row r="193" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A193" s="37">
@@ -8462,10 +8478,10 @@
         <f t="shared" ref="I193:I211" si="6">H193-G193</f>
         <v>0</v>
       </c>
-      <c r="J193" s="45"/>
-      <c r="K193" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J193" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K193" s="43"/>
     </row>
     <row r="194" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A194" s="37">
@@ -8496,10 +8512,10 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="J194" s="45"/>
-      <c r="K194" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J194" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K194" s="43"/>
     </row>
     <row r="195" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A195" s="37">
@@ -8562,7 +8578,7 @@
         <v>1.25</v>
       </c>
       <c r="J196" s="53" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="K196" s="43" t="s">
         <v>294</v>
@@ -8598,7 +8614,7 @@
         <v>1</v>
       </c>
       <c r="J197" s="53" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="K197" s="43"/>
     </row>
@@ -8664,7 +8680,7 @@
         <v>0</v>
       </c>
       <c r="J199" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K199" s="43"/>
     </row>
@@ -8698,7 +8714,7 @@
         <v>0</v>
       </c>
       <c r="J200" s="53" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K200" s="43"/>
     </row>
@@ -8732,7 +8748,7 @@
         <v>-0.5</v>
       </c>
       <c r="J201" s="53" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="K201" s="43"/>
     </row>
@@ -8898,7 +8914,7 @@
         <v>-0.5</v>
       </c>
       <c r="J206" s="53" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="K206" s="43" t="s">
         <v>318</v>
@@ -8934,7 +8950,7 @@
         <v>0.5</v>
       </c>
       <c r="J207" s="53" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="K207" s="43" t="s">
         <v>319</v>
@@ -8970,7 +8986,7 @@
         <v>2</v>
       </c>
       <c r="J208" s="53" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="K208" s="43" t="s">
         <v>350</v>
@@ -9005,10 +9021,10 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="J209" s="45"/>
-      <c r="K209" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J209" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K209" s="43"/>
     </row>
     <row r="210" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A210" s="37">
@@ -9039,10 +9055,10 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="J210" s="45"/>
-      <c r="K210" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J210" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K210" s="43"/>
     </row>
     <row r="211" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A211" s="13"/>
@@ -9069,53 +9085,53 @@
       <c r="K211" s="46"/>
     </row>
     <row r="212" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A212" s="74" t="s">
+      <c r="A212" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="B212" s="64"/>
-      <c r="C212" s="64"/>
-      <c r="D212" s="64"/>
-      <c r="E212" s="64"/>
-      <c r="F212" s="64"/>
-      <c r="G212" s="64"/>
-      <c r="H212" s="64"/>
-      <c r="I212" s="64"/>
-      <c r="J212" s="64"/>
-      <c r="K212" s="65"/>
+      <c r="B212" s="57"/>
+      <c r="C212" s="57"/>
+      <c r="D212" s="57"/>
+      <c r="E212" s="57"/>
+      <c r="F212" s="57"/>
+      <c r="G212" s="57"/>
+      <c r="H212" s="57"/>
+      <c r="I212" s="57"/>
+      <c r="J212" s="57"/>
+      <c r="K212" s="58"/>
     </row>
     <row r="213" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A213" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B213" s="71" t="s">
+      <c r="B213" s="77" t="s">
         <v>13</v>
       </c>
-      <c r="C213" s="64"/>
-      <c r="D213" s="64"/>
-      <c r="E213" s="64"/>
-      <c r="F213" s="64"/>
-      <c r="G213" s="64"/>
-      <c r="H213" s="64"/>
-      <c r="I213" s="64"/>
-      <c r="J213" s="64"/>
-      <c r="K213" s="65"/>
+      <c r="C213" s="57"/>
+      <c r="D213" s="57"/>
+      <c r="E213" s="57"/>
+      <c r="F213" s="57"/>
+      <c r="G213" s="57"/>
+      <c r="H213" s="57"/>
+      <c r="I213" s="57"/>
+      <c r="J213" s="57"/>
+      <c r="K213" s="58"/>
     </row>
     <row r="214" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A214" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B214" s="71" t="s">
+      <c r="B214" s="77" t="s">
         <v>15</v>
       </c>
-      <c r="C214" s="64"/>
-      <c r="D214" s="64"/>
-      <c r="E214" s="64"/>
-      <c r="F214" s="64"/>
-      <c r="G214" s="64"/>
-      <c r="H214" s="64"/>
-      <c r="I214" s="64"/>
-      <c r="J214" s="64"/>
-      <c r="K214" s="65"/>
+      <c r="C214" s="57"/>
+      <c r="D214" s="57"/>
+      <c r="E214" s="57"/>
+      <c r="F214" s="57"/>
+      <c r="G214" s="57"/>
+      <c r="H214" s="57"/>
+      <c r="I214" s="57"/>
+      <c r="J214" s="57"/>
+      <c r="K214" s="58"/>
     </row>
     <row r="215" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A215" s="37">
@@ -9146,10 +9162,10 @@
         <f t="shared" ref="I215:I235" si="7">H215-G215</f>
         <v>0</v>
       </c>
-      <c r="J215" s="45"/>
-      <c r="K215" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J215" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K215" s="43"/>
     </row>
     <row r="216" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A216" s="37">
@@ -9180,10 +9196,10 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J216" s="45"/>
-      <c r="K216" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J216" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K216" s="43"/>
     </row>
     <row r="217" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A217" s="37">
@@ -9342,10 +9358,10 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J221" s="45"/>
-      <c r="K221" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J221" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K221" s="43"/>
     </row>
     <row r="222" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A222" s="37">
@@ -9390,7 +9406,7 @@
         <v>315</v>
       </c>
       <c r="D223" s="38" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="E223" s="40" t="s">
         <v>63</v>
@@ -9409,7 +9425,7 @@
         <v>0</v>
       </c>
       <c r="J223" s="55" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="224" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -9442,7 +9458,7 @@
         <v>0</v>
       </c>
       <c r="J224" s="55" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="225" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -9475,7 +9491,7 @@
         <v>0</v>
       </c>
       <c r="J225" s="55" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="226" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -9507,10 +9523,10 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J226" s="45"/>
-      <c r="K226" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J226" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K226" s="43"/>
     </row>
     <row r="227" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A227" s="37">
@@ -9574,7 +9590,7 @@
         <v>0</v>
       </c>
       <c r="J228" s="55" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="229" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -9639,7 +9655,7 @@
         <v>1.75</v>
       </c>
       <c r="J230" s="53" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="K230" s="43" t="s">
         <v>351</v>
@@ -9675,7 +9691,7 @@
         <v>0.5</v>
       </c>
       <c r="J231" s="53" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="K231" s="43" t="s">
         <v>337</v>
@@ -9710,10 +9726,10 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J232" s="45"/>
-      <c r="K232" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J232" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K232" s="43"/>
     </row>
     <row r="233" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A233" s="37">
@@ -9744,10 +9760,10 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J233" s="45"/>
-      <c r="K233" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J233" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K233" s="43"/>
     </row>
     <row r="234" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A234" s="37">
@@ -9778,10 +9794,10 @@
         <f t="shared" si="7"/>
         <v>-0.15</v>
       </c>
-      <c r="J234" s="45"/>
-      <c r="K234" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J234" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K234" s="43"/>
     </row>
     <row r="235" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A235" s="13"/>
@@ -9808,53 +9824,53 @@
       <c r="K235" s="46"/>
     </row>
     <row r="236" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A236" s="56" t="s">
+      <c r="A236" s="64" t="s">
         <v>26</v>
       </c>
-      <c r="B236" s="57"/>
-      <c r="C236" s="57"/>
-      <c r="D236" s="57"/>
-      <c r="E236" s="57"/>
-      <c r="F236" s="57"/>
-      <c r="G236" s="57"/>
-      <c r="H236" s="57"/>
-      <c r="I236" s="57"/>
-      <c r="J236" s="57"/>
-      <c r="K236" s="58"/>
+      <c r="B236" s="65"/>
+      <c r="C236" s="65"/>
+      <c r="D236" s="65"/>
+      <c r="E236" s="65"/>
+      <c r="F236" s="65"/>
+      <c r="G236" s="65"/>
+      <c r="H236" s="65"/>
+      <c r="I236" s="65"/>
+      <c r="J236" s="65"/>
+      <c r="K236" s="66"/>
     </row>
     <row r="237" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A237" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B237" s="59" t="s">
+      <c r="B237" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="C237" s="57"/>
-      <c r="D237" s="57"/>
-      <c r="E237" s="57"/>
-      <c r="F237" s="57"/>
-      <c r="G237" s="57"/>
-      <c r="H237" s="57"/>
-      <c r="I237" s="57"/>
-      <c r="J237" s="57"/>
-      <c r="K237" s="58"/>
+      <c r="C237" s="65"/>
+      <c r="D237" s="65"/>
+      <c r="E237" s="65"/>
+      <c r="F237" s="65"/>
+      <c r="G237" s="65"/>
+      <c r="H237" s="65"/>
+      <c r="I237" s="65"/>
+      <c r="J237" s="65"/>
+      <c r="K237" s="66"/>
     </row>
     <row r="238" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A238" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B238" s="59" t="s">
+      <c r="B238" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="C238" s="57"/>
-      <c r="D238" s="57"/>
-      <c r="E238" s="57"/>
-      <c r="F238" s="57"/>
-      <c r="G238" s="57"/>
-      <c r="H238" s="57"/>
-      <c r="I238" s="57"/>
-      <c r="J238" s="57"/>
-      <c r="K238" s="58"/>
+      <c r="C238" s="65"/>
+      <c r="D238" s="65"/>
+      <c r="E238" s="65"/>
+      <c r="F238" s="65"/>
+      <c r="G238" s="65"/>
+      <c r="H238" s="65"/>
+      <c r="I238" s="65"/>
+      <c r="J238" s="65"/>
+      <c r="K238" s="66"/>
     </row>
     <row r="239" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A239" s="37">
@@ -9882,11 +9898,11 @@
         <v>0.5</v>
       </c>
       <c r="I239" s="41">
-        <f t="shared" ref="I239:I262" si="8">H239-G239</f>
+        <f t="shared" ref="I239:I264" si="8">H239-G239</f>
         <v>0</v>
       </c>
       <c r="J239" s="55" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="K239" s="43"/>
     </row>
@@ -9920,7 +9936,7 @@
         <v>0</v>
       </c>
       <c r="J240" s="53" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="K240" s="43"/>
     </row>
@@ -9954,7 +9970,7 @@
         <v>0</v>
       </c>
       <c r="J241" s="53" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="K241" s="43"/>
     </row>
@@ -10020,7 +10036,7 @@
         <v>0</v>
       </c>
       <c r="J243" s="53" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="K243" s="43"/>
     </row>
@@ -10053,10 +10069,10 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J244" s="45"/>
-      <c r="K244" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J244" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K244" s="43"/>
     </row>
     <row r="245" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A245" s="37">
@@ -10119,10 +10135,10 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J246" s="45"/>
-      <c r="K246" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J246" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="K246" s="43"/>
     </row>
     <row r="247" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A247" s="37">
@@ -10154,7 +10170,7 @@
         <v>0.25</v>
       </c>
       <c r="J247" s="53" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="K247" s="43" t="s">
         <v>352</v>
@@ -10190,7 +10206,7 @@
         <v>0</v>
       </c>
       <c r="J248" s="53" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="K248" s="43"/>
     </row>
@@ -10224,7 +10240,7 @@
         <v>0</v>
       </c>
       <c r="J249" s="53" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="K249" s="43"/>
     </row>
@@ -10258,7 +10274,7 @@
         <v>0</v>
       </c>
       <c r="J250" s="53" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="K250" s="43"/>
     </row>
@@ -10292,7 +10308,7 @@
         <v>0</v>
       </c>
       <c r="J251" s="53" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="K251" s="43"/>
     </row>
@@ -10326,7 +10342,7 @@
         <v>0</v>
       </c>
       <c r="J252" s="53" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="K252" s="43"/>
     </row>
@@ -10360,7 +10376,7 @@
         <v>0</v>
       </c>
       <c r="J253" s="53" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="K253" s="43"/>
     </row>
@@ -10375,7 +10391,7 @@
         <v>315</v>
       </c>
       <c r="D254" s="38" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="E254" s="40" t="s">
         <v>63</v>
@@ -10394,7 +10410,7 @@
         <v>0</v>
       </c>
       <c r="J254" s="53" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="K254" s="43"/>
     </row>
@@ -10427,10 +10443,10 @@
         <f t="shared" si="8"/>
         <v>0.10000000000000009</v>
       </c>
-      <c r="J255" s="45"/>
-      <c r="K255" s="43" t="s">
-        <v>365</v>
-      </c>
+      <c r="J255" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="K255" s="43"/>
     </row>
     <row r="256" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A256" s="37">
@@ -10443,7 +10459,7 @@
         <v>197</v>
       </c>
       <c r="D256" s="38" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="E256" s="40" t="s">
         <v>63</v>
@@ -10461,7 +10477,9 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J256" s="45"/>
+      <c r="J256" s="53" t="s">
+        <v>417</v>
+      </c>
       <c r="K256" s="43"/>
     </row>
     <row r="257" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -10469,29 +10487,33 @@
         <v>45680</v>
       </c>
       <c r="B257" s="38" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C257" s="39" t="s">
-        <v>197</v>
+        <v>79</v>
       </c>
       <c r="D257" s="38" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="E257" s="40" t="s">
         <v>63</v>
       </c>
       <c r="F257" s="40" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G257" s="41">
-        <v>1</v>
-      </c>
-      <c r="H257" s="41"/>
+        <v>0.15</v>
+      </c>
+      <c r="H257" s="41">
+        <v>0.15</v>
+      </c>
       <c r="I257" s="41">
         <f t="shared" si="8"/>
-        <v>-1</v>
-      </c>
-      <c r="J257" s="45"/>
+        <v>0</v>
+      </c>
+      <c r="J257" s="45" t="s">
+        <v>418</v>
+      </c>
       <c r="K257" s="43"/>
     </row>
     <row r="258" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
@@ -10502,10 +10524,10 @@
         <v>42</v>
       </c>
       <c r="C258" s="39" t="s">
-        <v>360</v>
+        <v>197</v>
       </c>
       <c r="D258" s="38" t="s">
-        <v>359</v>
+        <v>413</v>
       </c>
       <c r="E258" s="40" t="s">
         <v>63</v>
@@ -10514,12 +10536,12 @@
         <v>87</v>
       </c>
       <c r="G258" s="41">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H258" s="41"/>
       <c r="I258" s="41">
         <f t="shared" si="8"/>
-        <v>-0.5</v>
+        <v>-1</v>
       </c>
       <c r="J258" s="45"/>
       <c r="K258" s="43"/>
@@ -10532,98 +10554,158 @@
         <v>42</v>
       </c>
       <c r="C259" s="39" t="s">
-        <v>345</v>
+        <v>197</v>
       </c>
       <c r="D259" s="38" t="s">
-        <v>354</v>
+        <v>414</v>
       </c>
       <c r="E259" s="40" t="s">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="F259" s="40" t="s">
-        <v>348</v>
+        <v>87</v>
       </c>
       <c r="G259" s="41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H259" s="41"/>
       <c r="I259" s="41">
         <f t="shared" si="8"/>
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="J259" s="45"/>
       <c r="K259" s="43"/>
     </row>
     <row r="260" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A260" s="37"/>
-      <c r="B260" s="38"/>
+      <c r="A260" s="37">
+        <v>45680</v>
+      </c>
+      <c r="B260" s="38" t="s">
+        <v>42</v>
+      </c>
       <c r="C260" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D260" s="38"/>
-      <c r="E260" s="40"/>
-      <c r="F260" s="40"/>
-      <c r="G260" s="41"/>
+        <v>360</v>
+      </c>
+      <c r="D260" s="38" t="s">
+        <v>359</v>
+      </c>
+      <c r="E260" s="40" t="s">
+        <v>63</v>
+      </c>
+      <c r="F260" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G260" s="41">
+        <v>0.5</v>
+      </c>
       <c r="H260" s="41"/>
       <c r="I260" s="41">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="J260" s="45"/>
       <c r="K260" s="43"/>
     </row>
     <row r="261" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A261" s="37"/>
-      <c r="B261" s="38"/>
+      <c r="A261" s="37">
+        <v>45680</v>
+      </c>
+      <c r="B261" s="38" t="s">
+        <v>42</v>
+      </c>
       <c r="C261" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="D261" s="38"/>
-      <c r="E261" s="40"/>
-      <c r="F261" s="40"/>
-      <c r="G261" s="41"/>
+        <v>345</v>
+      </c>
+      <c r="D261" s="38" t="s">
+        <v>354</v>
+      </c>
+      <c r="E261" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="F261" s="40" t="s">
+        <v>348</v>
+      </c>
+      <c r="G261" s="41">
+        <v>2</v>
+      </c>
       <c r="H261" s="41"/>
       <c r="I261" s="41">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="J261" s="45"/>
       <c r="K261" s="43"/>
     </row>
     <row r="262" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A262" s="48"/>
-      <c r="B262" s="49"/>
-      <c r="C262" s="49"/>
-      <c r="D262" s="49"/>
-      <c r="E262" s="49" t="s">
+      <c r="A262" s="37"/>
+      <c r="B262" s="38"/>
+      <c r="C262" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D262" s="38"/>
+      <c r="E262" s="40"/>
+      <c r="F262" s="40"/>
+      <c r="G262" s="41"/>
+      <c r="H262" s="41"/>
+      <c r="I262" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J262" s="45"/>
+      <c r="K262" s="43"/>
+    </row>
+    <row r="263" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A263" s="37"/>
+      <c r="B263" s="38"/>
+      <c r="C263" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="D263" s="38"/>
+      <c r="E263" s="40"/>
+      <c r="F263" s="40"/>
+      <c r="G263" s="41"/>
+      <c r="H263" s="41"/>
+      <c r="I263" s="41">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J263" s="45"/>
+      <c r="K263" s="43"/>
+    </row>
+    <row r="264" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A264" s="48"/>
+      <c r="B264" s="49"/>
+      <c r="C264" s="49"/>
+      <c r="D264" s="49"/>
+      <c r="E264" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="F262" s="49"/>
-      <c r="G262" s="50">
-        <f t="shared" ref="G262:H262" si="9">SUM(G239:G261)</f>
-        <v>27.25</v>
-      </c>
-      <c r="H262" s="50">
+      <c r="F264" s="49"/>
+      <c r="G264" s="50">
+        <f t="shared" ref="G264:H264" si="9">SUM(G239:G263)</f>
+        <v>28.4</v>
+      </c>
+      <c r="H264" s="50">
         <f t="shared" si="9"/>
-        <v>24.1</v>
-      </c>
-      <c r="I262" s="50">
+        <v>24.25</v>
+      </c>
+      <c r="I264" s="50">
         <f t="shared" si="8"/>
-        <v>-3.1499999999999986</v>
-      </c>
-      <c r="J262" s="51"/>
-      <c r="K262" s="52"/>
-    </row>
-    <row r="263" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E263" s="40"/>
-    </row>
-    <row r="264" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G264" s="38" t="s">
+        <v>-4.1499999999999986</v>
+      </c>
+      <c r="J264" s="51"/>
+      <c r="K264" s="52"/>
+    </row>
+    <row r="265" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E265" s="40"/>
+    </row>
+    <row r="266" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G266" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="H264" s="54">
-        <f>H44+H79+H113+H146+H189+H211+H235+H262</f>
-        <v>251.68999999999997</v>
+      <c r="H266" s="54">
+        <f>H44+H79+H113+H146+H189+H211+H235+H264</f>
+        <v>251.83999999999997</v>
       </c>
     </row>
   </sheetData>
@@ -10631,7 +10713,7 @@
   <customSheetViews>
     <customSheetView guid="{8BAC9A6B-5D32-4E8D-967D-E17D357516F8}" filter="1" showAutoFilter="1">
       <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-      <autoFilter ref="A1:K15" xr:uid="{8E0EAE7C-0B36-4FA4-85FC-A2745880402C}">
+      <autoFilter ref="A1:K15" xr:uid="{CD1D9B45-343B-42EB-BF6B-FE134B2530F6}">
         <filterColumn colId="1">
           <filters blank="1">
             <filter val="- Weekplan item 1_x000a_- Weekplan item 2_x000a_- Weekplan item 3_x000a_- etc"/>
@@ -10642,14 +10724,6 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="24">
-    <mergeCell ref="B191:K191"/>
-    <mergeCell ref="B192:K192"/>
-    <mergeCell ref="A212:K212"/>
-    <mergeCell ref="B116:K116"/>
-    <mergeCell ref="A147:K147"/>
-    <mergeCell ref="B148:K148"/>
-    <mergeCell ref="B149:K149"/>
-    <mergeCell ref="A190:K190"/>
     <mergeCell ref="A236:K236"/>
     <mergeCell ref="B237:K237"/>
     <mergeCell ref="B238:K238"/>
@@ -10666,8 +10740,16 @@
     <mergeCell ref="B213:K213"/>
     <mergeCell ref="B214:K214"/>
     <mergeCell ref="B115:K115"/>
+    <mergeCell ref="B191:K191"/>
+    <mergeCell ref="B192:K192"/>
+    <mergeCell ref="A212:K212"/>
+    <mergeCell ref="B116:K116"/>
+    <mergeCell ref="A147:K147"/>
+    <mergeCell ref="B148:K148"/>
+    <mergeCell ref="B149:K149"/>
+    <mergeCell ref="A190:K190"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B43 B46:B78 B83:B112 B117:B145 B150:B188 B193:B210 B215:B234 B239:B261">
+  <conditionalFormatting sqref="B5:B43 B46:B78 B83:B112 B117:B145 B150:B188 B193:B210 B215:B234 B239:B263">
     <cfRule type="containsText" dxfId="10" priority="6" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -10684,7 +10766,7 @@
       <formula>NOT(ISERROR(SEARCH(("Done"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B44 B46:B79 B81:B113 B115:B146 B148:B189 B191:B211 B213:B235 B237:B262">
+  <conditionalFormatting sqref="B5:B44 B46:B79 B81:B113 B115:B146 B148:B189 B191:B211 B213:B235 B237:B264">
     <cfRule type="containsText" dxfId="5" priority="11" operator="containsText" text="Unplanned">
       <formula>NOT(ISERROR(SEARCH(("Unplanned"),(B5))))</formula>
     </cfRule>
@@ -10692,17 +10774,17 @@
       <formula>NOT(ISERROR(SEARCH(("Cancelled"),(B5))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1 G3:G44 G48:G79 G83:G113 G117:G146 G150:G189 G193:G211 G215:G235 G239:G262">
+  <conditionalFormatting sqref="G1 G3:G44 G48:G79 G83:G113 G117:G146 G150:G189 G193:G211 G215:G235 G239:G264">
     <cfRule type="cellIs" dxfId="3" priority="15" operator="greaterThan">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H262">
+  <conditionalFormatting sqref="H1:H264">
     <cfRule type="containsBlanks" dxfId="2" priority="16">
       <formula>LEN(TRIM(H1))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I44 I48:I79 I83:I113 I117:I146 I150:I189 I193:I211 I215:I235 I239:I262">
+  <conditionalFormatting sqref="I5:I44 I48:I79 I83:I113 I117:I146 I150:I189 I193:I211 I215:I235 I239:I264">
     <cfRule type="expression" dxfId="1" priority="13">
       <formula>H5/G5&gt;=1.5</formula>
     </cfRule>
@@ -10711,7 +10793,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F215:F234 F5:F43 F48:F78 F83:F112 F117:F145 F150:F188 F193:F210 F239:F261" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
+    <dataValidation type="list" allowBlank="1" sqref="F215:F234 F5:F43 F48:F78 F83:F112 F117:F145 F150:F188 F193:F210 F239:F263" xr:uid="{0FAB3063-668E-4727-8636-10D0A6594410}">
       <formula1>"ILO 0.2, ILO 1.2, ILO 2.2, ILO 6.2, ILO 8.1, ILO 8.2, ILO 11.1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10821,9 +10903,60 @@
     <hyperlink ref="J251" r:id="rId103" xr:uid="{16CA5873-1B08-42B1-8CFB-B21C99D3DA09}"/>
     <hyperlink ref="J248" r:id="rId104" xr:uid="{5579EECA-7B58-48DE-95CC-8A44F9E9CF3D}"/>
     <hyperlink ref="J247" r:id="rId105" xr:uid="{17750EDF-0632-423C-A63E-900EA839D2C0}"/>
+    <hyperlink ref="J15" r:id="rId106" xr:uid="{810C9D5C-DB19-4A50-B002-05E89C229713}"/>
+    <hyperlink ref="J18" r:id="rId107" xr:uid="{849433E2-2F89-4457-AE98-F2AD2E047E72}"/>
+    <hyperlink ref="J23" r:id="rId108" xr:uid="{F34838A9-C200-4A1A-8C44-12D0060E47C4}"/>
+    <hyperlink ref="J31" r:id="rId109" xr:uid="{5D7AE519-3FED-4484-906C-4DB6CC024995}"/>
+    <hyperlink ref="J41" r:id="rId110" xr:uid="{56880DEE-7FDC-4192-AC87-192B6976C29C}"/>
+    <hyperlink ref="J48" r:id="rId111" xr:uid="{E023C4C4-A2A5-4937-A80D-A21715F50902}"/>
+    <hyperlink ref="J77" r:id="rId112" xr:uid="{B7F7DCE1-43FD-410D-8DEB-B6EF37A4E012}"/>
+    <hyperlink ref="J83" r:id="rId113" xr:uid="{24AE4875-67F9-4D92-95C0-358302E7D8E4}"/>
+    <hyperlink ref="J92" r:id="rId114" xr:uid="{D8D58D01-EDEC-47F7-99EC-FFAFC30B863A}"/>
+    <hyperlink ref="J109" r:id="rId115" xr:uid="{CB5B7C5C-2590-46C6-BDE5-C76A0CF7E388}"/>
+    <hyperlink ref="J112" r:id="rId116" xr:uid="{EE16DA67-5141-4DDA-B82B-2CDDACFC7B42}"/>
+    <hyperlink ref="J118" r:id="rId117" xr:uid="{85E8E2BE-ABDD-47EE-9DC5-ACC82274FB23}"/>
+    <hyperlink ref="J138" r:id="rId118" xr:uid="{1AB57CC8-4C18-4DDD-A1E3-83248D7C98C3}"/>
+    <hyperlink ref="J145" r:id="rId119" xr:uid="{426B8A77-1352-4258-9169-76A1FB9C1888}"/>
+    <hyperlink ref="J150" r:id="rId120" xr:uid="{B050147F-68C8-40C8-B696-5DAB5E3A4CE2}"/>
+    <hyperlink ref="J167" r:id="rId121" xr:uid="{07AE4514-CDBB-4D2B-B81C-823A5841873F}"/>
+    <hyperlink ref="J169" r:id="rId122" xr:uid="{9D09B1CE-9462-4620-AC3E-DFF3DD606F48}"/>
+    <hyperlink ref="J177" r:id="rId123" xr:uid="{104D90F8-9682-4B2D-B5DF-362706681732}"/>
+    <hyperlink ref="J185" r:id="rId124" xr:uid="{5E0D6595-E405-46D3-89F8-05272038C703}"/>
+    <hyperlink ref="J187" r:id="rId125" xr:uid="{DEDDB964-A45C-4F77-A5A9-ED8B12693879}"/>
+    <hyperlink ref="J193" r:id="rId126" xr:uid="{879435ED-60FA-478E-A9CA-1AA53144C9C4}"/>
+    <hyperlink ref="J209" r:id="rId127" xr:uid="{D6C3E666-6286-4239-B523-E76DFBDE0824}"/>
+    <hyperlink ref="J215" r:id="rId128" xr:uid="{22C5F916-4608-4E13-A0DC-9F3146B165FC}"/>
+    <hyperlink ref="J221" r:id="rId129" xr:uid="{5B6501EE-C0CC-4509-8CC0-409E9F6DD34C}"/>
+    <hyperlink ref="J226" r:id="rId130" xr:uid="{C03DA8D6-7673-48F5-9285-42BB17C9E10A}"/>
+    <hyperlink ref="J234" r:id="rId131" xr:uid="{E3781C19-A3A7-417B-9AF6-1A4B5C29ED49}"/>
+    <hyperlink ref="J244" r:id="rId132" xr:uid="{E8EBB20C-64B8-4D8A-809D-C7782713810C}"/>
+    <hyperlink ref="J255" r:id="rId133" xr:uid="{4CD52B8B-666A-4810-8891-B9701AF47292}"/>
+    <hyperlink ref="J42" r:id="rId134" xr:uid="{9E2DBD53-1B37-4AFD-9D09-C80AD2CED5F3}"/>
+    <hyperlink ref="J43" r:id="rId135" xr:uid="{6911F2DF-A958-4D75-996E-C60149131810}"/>
+    <hyperlink ref="J55" r:id="rId136" xr:uid="{B4CA1D2D-3394-48DC-AFD5-8996A98BAC15}"/>
+    <hyperlink ref="J74" r:id="rId137" xr:uid="{79EACBE7-45A2-46C7-BF9B-D3B6F1C2C7A0}"/>
+    <hyperlink ref="J75" r:id="rId138" xr:uid="{2E7CD377-C748-441B-8BA0-B3E1C11185DB}"/>
+    <hyperlink ref="J76" r:id="rId139" xr:uid="{D6C45377-08A1-4A88-8581-7729E845289C}"/>
+    <hyperlink ref="J78" r:id="rId140" xr:uid="{3C15A722-14F1-4100-B14C-2B694A08BF87}"/>
+    <hyperlink ref="J84" r:id="rId141" xr:uid="{AE0416F3-33B3-4A14-A0E1-5CFBDE104FA2}"/>
+    <hyperlink ref="J110" r:id="rId142" xr:uid="{FF91C10D-6466-41F0-B06E-0A0A1698C653}"/>
+    <hyperlink ref="J111" r:id="rId143" xr:uid="{6A0D7A34-A3D1-473B-9F18-27B3400E2CFB}"/>
+    <hyperlink ref="J117" r:id="rId144" xr:uid="{DF77F81A-B1FF-4A7F-9573-BD0346A42F53}"/>
+    <hyperlink ref="J143" r:id="rId145" xr:uid="{2F4BB9AA-AB86-4677-8BBD-E6FF8064E007}"/>
+    <hyperlink ref="J144" r:id="rId146" xr:uid="{639D621D-8894-468B-9237-CF6D52BFBD30}"/>
+    <hyperlink ref="J151" r:id="rId147" xr:uid="{06D8DA03-C223-4C8E-B470-1285C28FB832}"/>
+    <hyperlink ref="J186" r:id="rId148" xr:uid="{B1689ADF-32FF-4C14-A28A-DD9614EB5B69}"/>
+    <hyperlink ref="J188" r:id="rId149" xr:uid="{26C4B599-CD6E-4FFE-BB34-765E8798BA5B}"/>
+    <hyperlink ref="J210" r:id="rId150" xr:uid="{D4094CB6-1C9D-4B70-A589-15ABA37B9022}"/>
+    <hyperlink ref="J194" r:id="rId151" xr:uid="{BDC74E4A-FF09-47DE-9FE2-69AFEFB1275F}"/>
+    <hyperlink ref="J216" r:id="rId152" xr:uid="{5FD21133-56B1-4C02-86BA-BF3DFE230C7B}"/>
+    <hyperlink ref="J232" r:id="rId153" xr:uid="{4094066C-DC72-4BE3-8460-4E275C703158}"/>
+    <hyperlink ref="J233" r:id="rId154" xr:uid="{11DEE17A-3989-4545-AEDA-52271259F45E}"/>
+    <hyperlink ref="J246" r:id="rId155" xr:uid="{213A3762-904B-4D21-817E-12DF4A085F48}"/>
+    <hyperlink ref="J256" r:id="rId156" xr:uid="{0B4B23F4-04E5-496C-BF6B-0D3C4A045F03}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="52" fitToHeight="0" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId106"/>
+  <pageSetup paperSize="9" scale="52" fitToHeight="0" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId157"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
@@ -10831,13 +10964,13 @@
           <x14:formula1>
             <xm:f>'Drop-downs'!$B$2:$B$16</xm:f>
           </x14:formula1>
-          <xm:sqref>E215:E234 E5:E43 E48:E78 E83:E112 E117:E145 E150:E188 E193:E210 E239:E261</xm:sqref>
+          <xm:sqref>E215:E234 E5:E43 E48:E78 E83:E112 E117:E145 E150:E188 E193:E210 E239:E263</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Drop-downs'!$A$2:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>B215:B234 B5:B43 B48:B78 B83:B112 B117:B145 B150:B188 B193:B210 B239:B261</xm:sqref>
+          <xm:sqref>B215:B234 B5:B43 B48:B78 B83:B112 B117:B145 B150:B188 B193:B210 B239:B263</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -12478,6 +12611,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000BADAD4AA324BF48804EF76FD903323C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4ea0feda506421460444ca95554a0aab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5ff92c65-ed86-4457-baee-ccd535c9ea21" xmlns:ns3="6c8d291c-a5bf-4049-930d-38db8e991d8e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0fc8cf7d0f5ee312899395875a30595e" ns2:_="" ns3:_="">
     <xsd:import namespace="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
@@ -12712,27 +12865,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="6c8d291c-a5bf-4049-930d-38db8e991d8e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5ff92c65-ed86-4457-baee-ccd535c9ea21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
+    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBBEA8C5-7A8E-4EDD-924F-588BDEE1426F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12749,23 +12901,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{320CF63A-30C9-4A8C-8DF9-EA62B8EC1A62}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6c8d291c-a5bf-4049-930d-38db8e991d8e"/>
-    <ds:schemaRef ds:uri="5ff92c65-ed86-4457-baee-ccd535c9ea21"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A64A65-7DA4-4AE1-9847-B817073E4705}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>